<commit_message>
Cottage Grove and Dorena evac rates were mixed up
</commit_message>
<xml_diff>
--- a/data/common_data/Reservoirs.xlsx
+++ b/data/common_data/Reservoirs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Python\Willamette_FIRO\data\common_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A21550-59BE-4A66-83F8-E494AB2CA51F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D6E9153-EED6-4EFD-B753-1353D73E6655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-84" windowWidth="23256" windowHeight="13872" xr2:uid="{FC561D18-D4CD-4EFF-9AED-16460E500202}"/>
+    <workbookView xWindow="30120" yWindow="3105" windowWidth="21600" windowHeight="11280" xr2:uid="{FC561D18-D4CD-4EFF-9AED-16460E500202}"/>
   </bookViews>
   <sheets>
     <sheet name="Reservoirs" sheetId="2" r:id="rId1"/>
@@ -863,43 +863,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DBC2FD2-6A64-426A-9430-3B333C72098D}">
   <dimension ref="A1:P20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.6640625" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" customWidth="1"/>
-    <col min="5" max="11" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" customWidth="1"/>
+    <col min="5" max="11" width="14.42578125" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="14.88671875" customWidth="1"/>
-    <col min="14" max="15" width="16.109375" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" customWidth="1"/>
+    <col min="14" max="15" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -949,7 +949,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1</v>
       </c>
@@ -992,7 +992,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>4</v>
       </c>
@@ -1109,10 +1109,10 @@
         <v>835</v>
       </c>
       <c r="L10" s="1">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="M10" s="1">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="N10" s="1">
         <v>791</v>
@@ -1121,7 +1121,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5</v>
       </c>
@@ -1151,10 +1151,10 @@
         <v>791</v>
       </c>
       <c r="L11" s="1">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="M11" s="1">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="N11" s="1">
         <v>835</v>
@@ -1163,7 +1163,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>8</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>11</v>
       </c>
@@ -1415,7 +1415,11 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K20" s="1"/>
     </row>
   </sheetData>

</xml_diff>